<commit_message>
avances en el informe (revisar)deje coloreado en azul
</commit_message>
<xml_diff>
--- a/DSY1104 Evaluación Parcial 1 - Anexo 2 Planilla de Requerimientos.xlsx
+++ b/DSY1104 Evaluación Parcial 1 - Anexo 2 Planilla de Requerimientos.xlsx
@@ -1,27 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sj-alumno\Desktop\a\Proyecto-Fullstack-II\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moka/Documents/Fullstack II/Proyecto-Fullstack-II/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB76059-4F91-46CD-AFF6-FFE439DD94B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA22DD5C-8ACC-964B-9630-FF00825923DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="450" windowWidth="29040" windowHeight="15150" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="29040" windowHeight="15160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="4" r:id="rId1"/>
     <sheet name="Requerimiento Inicial" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -406,20 +401,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -429,8 +424,8 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -712,13 +707,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="41.85546875" customWidth="1"/>
-    <col min="2" max="2" width="150.42578125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="41.83203125" customWidth="1"/>
+    <col min="2" max="2" width="150.5" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="22" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>20</v>
       </c>
@@ -726,7 +721,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="37.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="20" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -734,7 +729,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="40" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>18</v>
       </c>
@@ -742,7 +737,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="20" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>32</v>
       </c>
@@ -750,7 +745,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="20" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>1</v>
       </c>
@@ -758,7 +753,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="60" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>19</v>
       </c>
@@ -766,7 +761,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>27</v>
       </c>
@@ -774,7 +769,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>26</v>
       </c>
@@ -791,18 +786,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.140625" customWidth="1"/>
-    <col min="2" max="2" width="35.42578125" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" customWidth="1"/>
-    <col min="4" max="4" width="29.28515625" customWidth="1"/>
-    <col min="5" max="5" width="28.7109375" customWidth="1"/>
-    <col min="6" max="6" width="108.85546875" customWidth="1"/>
-    <col min="7" max="7" width="28.42578125" customWidth="1"/>
+    <col min="1" max="1" width="8.1640625" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" customWidth="1"/>
+    <col min="4" max="4" width="29.33203125" customWidth="1"/>
+    <col min="5" max="5" width="28.6640625" customWidth="1"/>
+    <col min="6" max="6" width="108.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -825,7 +820,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
@@ -845,10 +840,10 @@
         <v>78</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
         <v>4</v>
       </c>
@@ -871,7 +866,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
         <v>5</v>
       </c>
@@ -894,7 +889,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>6</v>
       </c>
@@ -917,7 +912,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>7</v>
       </c>
@@ -940,7 +935,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>8</v>
       </c>
@@ -963,7 +958,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>9</v>
       </c>
@@ -986,7 +981,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>10</v>
       </c>
@@ -1009,7 +1004,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>11</v>
       </c>
@@ -1032,7 +1027,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
         <v>12</v>
       </c>
@@ -1052,10 +1047,10 @@
         <v>52</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>13</v>
       </c>
@@ -1078,7 +1073,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
         <v>14</v>
       </c>
@@ -1101,7 +1096,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>15</v>
       </c>
@@ -1124,7 +1119,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
         <v>16</v>
       </c>
@@ -1144,10 +1139,10 @@
         <v>73</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>17</v>
       </c>
@@ -1167,10 +1162,10 @@
         <v>72</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="22" spans="7:7" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="7:7" x14ac:dyDescent="0.2">
       <c r="G22" s="10"/>
     </row>
   </sheetData>
@@ -1180,15 +1175,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005395107FFD641345A10C8A5ACACB9D20" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ce7786e0ad11988b1588e06b80e33958">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e1e7bc46-bed0-459f-9452-a76b1c5b695e" xmlns:ns3="bb8cf7e1-610f-40a0-8f00-126b9d139fde" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="99ef8fa6ee73c11c731191fdf3d87e67" ns2:_="" ns3:_="">
     <xsd:import namespace="e1e7bc46-bed0-459f-9452-a76b1c5b695e"/>
@@ -1399,6 +1385,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1410,14 +1405,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{370A914A-1DD7-4F78-8671-F61C286C2CC1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F4FA5F9-E1BF-40AC-BEF4-FE15B10C9F42}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1436,6 +1423,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{370A914A-1DD7-4F78-8671-F61C286C2CC1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14168F1D-C031-4047-A789-A93363341739}">
   <ds:schemaRefs>

</xml_diff>